<commit_message>
Regenerate sales CRM workbook [skip crm]
</commit_message>
<xml_diff>
--- a/sales-engine/Same-Day-Customer-Growth-Pack-Live-CRM.xlsx
+++ b/sales-engine/Same-Day-Customer-Growth-Pack-Live-CRM.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="224">
   <si>
     <t>Rank</t>
   </si>
@@ -72,19 +72,60 @@
     <t>Status</t>
   </si>
   <si>
+    <t>Therma Tech</t>
+  </si>
+  <si>
+    <t>HVAC</t>
+  </si>
+  <si>
+    <t>San Jose, CA</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Official contact page is current: Mon–Fri 7:00 AM–5:30 PM, info@thermatechhvac.com, and a stated reply within 1 business hour. Current site also promotes flexible financing for new systems.</t>
+  </si>
+  <si>
+    <t>(408) 629-5400</t>
+  </si>
+  <si>
+    <t>info@thermatechhvac.com</t>
+  </si>
+  <si>
+    <t>Monday open; email reply target within 1 business hour</t>
+  </si>
+  <si>
+    <t>Turn financing and same-day HVAC decision friction into plain-English cost/option education.</t>
+  </si>
+  <si>
+    <t>Idea for Therma Tech’s financing traffic</t>
+  </si>
+  <si>
+    <t>Hi — I checked Therma Tech’s current financing and contact pages today and noticed you publish a one-business-hour email response target.
+I think there’s a strong customer question to build around:
+“Can I solve the HVAC problem now without taking the entire replacement cost at once?”
+I’d turn that into financing FAQs, Google/social posts, estimate follow-ups, objection responses and customer reactivation copy.
+Same-Day Customer Growth Pack: $150 flat, no subscription.
+Want me to send two Therma Tech-specific examples first?</t>
+  </si>
+  <si>
+    <t>https://thermatechhvac.com/contact</t>
+  </si>
+  <si>
+    <t>2026-09-07</t>
+  </si>
+  <si>
+    <t>Contact Ready</t>
+  </si>
+  <si>
     <t>Leader Restoration</t>
   </si>
   <si>
     <t>Mold / Water / Fire Restoration</t>
   </si>
   <si>
-    <t>San Jose, CA</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>September 2026 FREE mold inspection is live through Sep 30; 24/7 emergency response; published 60-minute arrival target; official site publishes service@leaderestoration.com.</t>
+    <t>September 2026 FREE mold inspection remains live through Sep 30. The official campaign publishes 24/7 response, 60-minute arrival target, service@leaderestoration.com, and direct insurance billing.</t>
   </si>
   <si>
     <t>(408) 868-2433</t>
@@ -93,10 +134,10 @@
     <t>service@leaderestoration.com</t>
   </si>
   <si>
-    <t>24/7</t>
-  </si>
-  <si>
-    <t>Use the expiring September inspection offer as education about hidden moisture/mold rather than generic discount advertising.</t>
+    <t>24/7; direct email</t>
+  </si>
+  <si>
+    <t>Use the expiring September inspection as customer education about hidden moisture and mold risk.</t>
   </si>
   <si>
     <t>2 ideas for your September mold-inspection campaign</t>
@@ -107,25 +148,19 @@
 “You don’t need visible mold to have a moisture problem worth investigating.”
 I’d turn that into a complete September campaign: Google/social posts, homeowner FAQs, inspection reminders, customer follow-ups and genuine review-request copy.
 Same-Day Customer Growth Pack: $150 flat, no subscription.
-I already drafted two more Leader-specific examples. Want me to send them?</t>
+I already drafted two Leader-specific examples. Want me to send them?</t>
   </si>
   <si>
     <t>https://call.leaderestoration.com/mold-408</t>
   </si>
   <si>
-    <t>2026-09-06</t>
-  </si>
-  <si>
-    <t>Contact Ready</t>
-  </si>
-  <si>
     <t>FloodDry Water Damage Restoration</t>
   </si>
   <si>
     <t>Water / Mold Restoration</t>
   </si>
   <si>
-    <t>Official site is current today: 24/7 emergency response, free inspections, ~45-minute on-site target, direct email, and recent customer reviews posted within the last week.</t>
+    <t>Official San Jose page was crawled today and publishes 24/7 emergency response, free inspections, roughly 45-minute response in many ZIP codes, moisture mapping/documentation, and service@flooddrywdr.com. Contact page shows customer reviews from 3 and 5 days ago.</t>
   </si>
   <si>
     <t>(408) 404-4000</t>
@@ -134,7 +169,10 @@
     <t>service@flooddrywdr.com</t>
   </si>
   <si>
-    <t>Translate moisture mapping, drying logs and insurance documentation into plain-English emergency education.</t>
+    <t>24/7; direct email; recent customer activity</t>
+  </si>
+  <si>
+    <t>Translate moisture mapping, drying logs and insurance documentation into urgent plain-English education.</t>
   </si>
   <si>
     <t>Customer-education idea for FloodDry’s free inspection</t>
@@ -142,13 +180,50 @@
   <si>
     <t>Hi — I reviewed FloodDry’s current San Jose service process today and found a strong customer-education angle:
 “The floor can look dry while moisture is still inside the structure.”
-Your published process already supports that message with moisture readings, structural drying and insurance documentation.
+Your published process already supports that message with moisture readings, structural drying, drying logs and insurance documentation.
 I’d turn it into emergency Google/social posts, homeowner FAQs, inspection follow-ups, insurance-documentation reminders and genuine review-request copy.
 Complete Same-Day Customer Growth Pack: $150 flat.
 Want me to send two FloodDry-specific samples first?</t>
   </si>
   <si>
-    <t>https://flooddrywdr.com/</t>
+    <t>https://flooddrywdr.com/water-damage-restoration-san-jose/</t>
+  </si>
+  <si>
+    <t>ROOF EXPRESS</t>
+  </si>
+  <si>
+    <t>Roofing</t>
+  </si>
+  <si>
+    <t>San Jose / Bay Area, CA</t>
+  </si>
+  <si>
+    <t>Official contact page publishes sales@roof-ex.com, phone/WhatsApp responses typically within minutes during business hours, free no-obligation roof inspections, and email replies within one business day. Current San Jose page adds photo documentation, financing up to $25,000 and 24/7 emergency roofing.</t>
+  </si>
+  <si>
+    <t>(650) 666-5554</t>
+  </si>
+  <si>
+    <t>sales@roof-ex.com</t>
+  </si>
+  <si>
+    <t>Mon–Fri 7–7; phone/WhatsApp typically answered within minutes</t>
+  </si>
+  <si>
+    <t>Market the transparent inspection → photo evidence → line-item scope → financing decision path.</t>
+  </si>
+  <si>
+    <t>Idea for ROOF EXPRESS’s inspection-to-estimate flow</t>
+  </si>
+  <si>
+    <t>Hi — I reviewed ROOF EXPRESS’s current San Jose and contact pages today. Your inspection process gives you a stronger customer story than another generic roofing ad:
+“See what the roof needs, what it costs and what the financing options are before deciding.”
+I’d turn that into inspection posts, financing FAQs, estimate follow-ups, repair-vs-replacement education and genuine review-request copy.
+Complete Same-Day Customer Growth Pack: $150 flat.
+Want two ROOF EXPRESS-specific examples first?</t>
+  </si>
+  <si>
+    <t>https://quote.roof-ex.com/contact/</t>
   </si>
   <si>
     <t>IRBIS Air Plumbing Electrical</t>
@@ -157,22 +232,22 @@
     <t>HVAC / Plumbing / Electrical</t>
   </si>
   <si>
-    <t>Official site crawled today advertises same-day service across HVAC, plumbing and electrical, seven days a week; current business listing shows 24/7 operation and 942 reviews.</t>
-  </si>
-  <si>
-    <t>(669) 266-5464</t>
-  </si>
-  <si>
-    <t>Same-day / 7 days</t>
-  </si>
-  <si>
-    <t>Build one-home-one-team messaging around multiple urgent trades and same-day availability.</t>
+    <t>Official site was crawled yesterday and promotes same-day San Jose HVAC/plumbing/electrical service, 40+ trucks, free estimates, and Monday-Friday same-day dispatch with a 24/7 support line. A current official rebate page publishes (408) 317-3901.</t>
+  </si>
+  <si>
+    <t>(408) 317-3901</t>
+  </si>
+  <si>
+    <t>Monday same-day service; 24/7 support line</t>
+  </si>
+  <si>
+    <t>Build one-home-one-team messaging around problems that cross HVAC, plumbing and electrical.</t>
   </si>
   <si>
     <t>One campaign across HVAC + plumbing + electrical</t>
   </si>
   <si>
-    <t>Hi — I was reviewing IRBIS today and your biggest marketing advantage isn’t one individual service — it’s that one team can handle HVAC, plumbing and electrical with same-day availability.
+    <t>Hi — I reviewed IRBIS today and your strongest marketing advantage isn’t one individual trade — it’s that HVAC, plumbing and electrical sit under one team.
 Campaign angle:
 “One call when the problem crosses systems.”
 I’d turn that into same-day service posts, cross-service homeowner FAQs, missed-inquiry follow-ups, estimate follow-ups and genuine review-request messaging.
@@ -189,13 +264,16 @@
     <t>Water / Fire / Mold / Reconstruction</t>
   </si>
   <si>
-    <t>Official San Jose page advertises 24/7 live dispatch, local 45-minute response target, direct insurance billing, $0 upfront on covered claims, and full restoration/reconstruction.</t>
+    <t>Official San Jose page advertises 24/7 live dispatch, a 45-minute local response target, free inspection, direct insurance billing, no upfront cost on covered claims, and restoration through reconstruction.</t>
   </si>
   <si>
     <t>(408) 402-4941</t>
   </si>
   <si>
-    <t>Turn emergency response + insurance handling + rebuild capability into a clear first-call workflow.</t>
+    <t>24/7 live dispatch</t>
+  </si>
+  <si>
+    <t>Turn emergency response + insurance handling + rebuild capability into one clear first-call workflow.</t>
   </si>
   <si>
     <t>San Jose restoration campaign idea</t>
@@ -211,6 +289,40 @@
     <t>https://cawaterandfire.com/san-jose/</t>
   </si>
   <si>
+    <t>Lifetime Roofing &amp; Renovation, Inc.</t>
+  </si>
+  <si>
+    <t>Roofing / Exterior Renovation</t>
+  </si>
+  <si>
+    <t>Sunnyvale / San Jose, CA</t>
+  </si>
+  <si>
+    <t>Official site was crawled yesterday and publishes free inspections, same-day roof inspections, Mon–Sat 8 AM–8 PM, emergency calls 24/7, 50-year warranty availability, and roofs starting at $12,000.</t>
+  </si>
+  <si>
+    <t>(408) 685-2177</t>
+  </si>
+  <si>
+    <t>Monday 8 AM–8 PM; emergency calls 24/7</t>
+  </si>
+  <si>
+    <t>Use same-day inspections and high-ticket roof decisions to create a pre-rain inspection + estimate follow-up sequence.</t>
+  </si>
+  <si>
+    <t>Idea for Lifetime’s same-day inspection campaign</t>
+  </si>
+  <si>
+    <t>Hi — I checked Lifetime’s current San Jose roofing page today and your same-day inspection offer gives you a strong customer campaign:
+“The first rain shouldn’t be the first time you learn where the roof is vulnerable.”
+I’d turn that into roof-and-drainage education, Google/social posts, inspection reminders, estimate follow-ups and repair-vs-replacement FAQs.
+Same-Day Customer Growth Pack: $150 flat.
+Want two Lifetime-specific examples first?</t>
+  </si>
+  <si>
+    <t>https://lifetimeroofingrenovation.com/</t>
+  </si>
+  <si>
     <t>Infinium Solar, Roofing and Electric</t>
   </si>
   <si>
@@ -220,13 +332,13 @@
     <t>Campbell / San Jose, CA</t>
   </si>
   <si>
-    <t>Official site is current today and combines solar, roofing and electrical in-house; Campbell/San Jose phone is published; services include battery, roof replacement, panel upgrades and EV charging.</t>
+    <t>Official pages remain current and combine solar, roofing and electrical under one contractor, with free estimates and a Campbell contact number. Current business listing shows Monday hours through 7 PM.</t>
   </si>
   <si>
     <t>(408) 583-8101</t>
   </si>
   <si>
-    <t>Sunday availability shown in current business listing</t>
+    <t>Monday; official Campbell line; current listing open through 7 PM</t>
   </si>
   <si>
     <t>Use pre-solar roof/electrical readiness and bundled project coordination as the campaign.</t>
@@ -242,78 +354,38 @@
 Want two Infinium-specific samples first?</t>
   </si>
   <si>
-    <t>https://infinium.inc/</t>
-  </si>
-  <si>
-    <t>Lifetime Roofing &amp; Renovation, Inc.</t>
-  </si>
-  <si>
-    <t>Roofing / Exterior Renovation</t>
-  </si>
-  <si>
-    <t>Sunnyvale / San Jose, CA</t>
-  </si>
-  <si>
-    <t>Official site advertises free/same-day inspections, 24/7 emergency service, San Jose coverage, and a current September storm-readiness inspection campaign ahead of rainy season.</t>
-  </si>
-  <si>
-    <t>(408) 685-2177</t>
-  </si>
-  <si>
-    <t>Emergency 24/7; regular Mon–Sat</t>
-  </si>
-  <si>
-    <t>Turn free storm-readiness inspections into a pre-rain roof + drainage education sequence.</t>
-  </si>
-  <si>
-    <t>Idea for Lifetime’s September inspection campaign</t>
-  </si>
-  <si>
-    <t>Hi — I checked Lifetime’s current September roof-inspection messaging and there’s a strong campaign hiding inside the offer:
-“The first rain shouldn’t be the first time you learn where the roof is vulnerable.”
-I’d turn the free inspection into roof-and-drainage education, Google/social posts, inspection reminders, estimate follow-ups and repair-vs-replacement FAQs.
+    <t>https://infinium.inc/campbell-ca/</t>
+  </si>
+  <si>
+    <t>Eastman Roofing &amp; Waterproofing, Inc.</t>
+  </si>
+  <si>
+    <t>Roofing / Waterproofing</t>
+  </si>
+  <si>
+    <t>Official site was crawled within the last week and promotes free estimates, emergency leak help, financing, repair-vs-replacement education, detailed written quotes, and 100% roof-replacement financing. Monday hours are 8:30 AM–5 PM.</t>
+  </si>
+  <si>
+    <t>(408) 971-9000</t>
+  </si>
+  <si>
+    <t>Monday 8:30 AM–5 PM</t>
+  </si>
+  <si>
+    <t>Turn its explicit “we won’t sell you a roof you don’t need” positioning into a repair-vs-replacement trust campaign.</t>
+  </si>
+  <si>
+    <t>Repair-vs-replacement campaign idea for Eastman</t>
+  </si>
+  <si>
+    <t>Hi — I reviewed Eastman’s current site today and your “we won’t sell you a roof you don’t need” pledge is a strong campaign idea on its own:
+“Before replacing the roof, find out whether the problem can actually be repaired.”
+I’d turn that into repair-vs-replacement FAQs, inspection education, financing objection responses, estimate follow-ups and homeowner trust content.
 Same-Day Customer Growth Pack: $150 flat.
-Want two Lifetime-specific examples first?</t>
-  </si>
-  <si>
-    <t>https://lifetimeroofingrenovation.com/</t>
-  </si>
-  <si>
-    <t>ROOF EXPRESS</t>
-  </si>
-  <si>
-    <t>Roofing</t>
-  </si>
-  <si>
-    <t>San Jose / Bay Area, CA</t>
-  </si>
-  <si>
-    <t>Official site is current today: free estimates, same-day inspections Mon–Sat, photo-supported line-item scopes within 24 hours, financing up to $25,000, 24/7 emergency service, and sales@roof-ex.com.</t>
-  </si>
-  <si>
-    <t>(650) 666-5554</t>
-  </si>
-  <si>
-    <t>sales@roof-ex.com</t>
-  </si>
-  <si>
-    <t>Emergency 24/7; Sunday by appointment</t>
-  </si>
-  <si>
-    <t>Sell the transparent inspection → photo scope → financing decision process rather than generic roofing.</t>
-  </si>
-  <si>
-    <t>Idea for ROOF EXPRESS’s inspection-to-estimate flow</t>
-  </si>
-  <si>
-    <t>Hi — I reviewed ROOF EXPRESS today and your inspection process gives you a better customer story than a generic roofing ad:
-“See what the roof needs, what it costs and what the financing options are before deciding.”
-I’d build that into inspection posts, financing FAQs, estimate follow-ups, repair-vs-replacement education and genuine review-request copy.
-Complete Same-Day Customer Growth Pack: $150 flat.
-Want two ROOF EXPRESS-specific examples first?</t>
-  </si>
-  <si>
-    <t>https://roof-ex.com/san-jose</t>
+Want two Eastman-specific examples first?</t>
+  </si>
+  <si>
+    <t>https://www.eastmanroofing.com/</t>
   </si>
   <si>
     <t>Any Hour Water and Fire</t>
@@ -325,23 +397,22 @@
     <t>San Jose area</t>
   </si>
   <si>
-    <t>Current business listing shows Sunday hours 8 AM–5 PM, 5.0 rating with 296 reviews, and emergency mitigation/cleanup/rebuild positioning.</t>
+    <t>Current business listing shows Monday 8 AM–5 PM, a 5.0 rating with 296 reviews, and emergency mitigation, drying, cleanup and rebuild positioning.</t>
   </si>
   <si>
     <t>(669) 304-3545</t>
   </si>
   <si>
-    <t>Sunday 8:00–5:00</t>
-  </si>
-  <si>
-    <t>Lead with mitigation-first education before rebuild and insurance complexity.</t>
+    <t>Monday 8 AM–5 PM</t>
+  </si>
+  <si>
+    <t>Lead with mitigation-first education before reconstruction and insurance complexity.</t>
   </si>
   <si>
     <t>Mitigation-first campaign idea</t>
   </si>
   <si>
-    <t>Hi — I was refreshing San Jose restoration companies today and Any Hour stood out because you’re actually reachable on Sunday.
-Campaign angle:
+    <t>Hi — I was refreshing San Jose restoration companies today and Any Hour stood out for a simple customer-education campaign:
 “Before worrying about rebuilding, stop the damage that’s still happening.”
 I’d turn that into a first-response checklist, mitigation FAQs, emergency Google/social posts, customer follow-ups and genuine review-request copy.
 Same-Day Customer Growth Pack: $150 flat.
@@ -349,68 +420,6 @@
   </si>
   <si>
     <t>https://www.google.com/search?q=Any+Hour+Water+and+Fire+San+Jose</t>
-  </si>
-  <si>
-    <t>South Bay Roofing CO</t>
-  </si>
-  <si>
-    <t>Official site updated within days: free inspection, roof/attic/flashing/gutter assessment, same-day itemized written quote, financing options and emergency roofing calls anytime.</t>
-  </si>
-  <si>
-    <t>(650) 447-1464</t>
-  </si>
-  <si>
-    <t>Emergency calls anytime; regular Mon–Sat</t>
-  </si>
-  <si>
-    <t>Use the no-pressure inspection + same-day itemized quote as a trust/decision campaign.</t>
-  </si>
-  <si>
-    <t>Turn your same-day roofing quote into a follow-up system</t>
-  </si>
-  <si>
-    <t>Hi — I reviewed South Bay Roofing’s current San Jose process and think the best campaign is already inside the way you sell:
-“Free inspection. Same-day itemized quote. No-pressure decision.”
-I’d turn that into inspection education, estimate follow-ups, repair-vs-replacement FAQs, financing objection responses and seasonal Google/social posts.
-Complete Same-Day Customer Growth Pack: $150 flat.
-Want two South Bay Roofing-specific examples first?</t>
-  </si>
-  <si>
-    <t>https://www.southbayroofingco.com/</t>
-  </si>
-  <si>
-    <t>Therma Tech</t>
-  </si>
-  <si>
-    <t>HVAC</t>
-  </si>
-  <si>
-    <t>Official pages remain current: financing subject to approval, free estimates, direct email with stated one-business-hour reply, plus a current same-day-service landing page crawled today.</t>
-  </si>
-  <si>
-    <t>(408) 629-5400</t>
-  </si>
-  <si>
-    <t>info@thermatechhvac.com</t>
-  </si>
-  <si>
-    <t>Regular office closed Sunday; same-day landing page active</t>
-  </si>
-  <si>
-    <t>Combine financing and same-day repair/installation messaging into plain-English decision support.</t>
-  </si>
-  <si>
-    <t>Idea for Therma Tech’s financing + same-day traffic</t>
-  </si>
-  <si>
-    <t>Hi — I checked Therma Tech’s current financing and same-day service pages today and there’s a useful customer question connecting both:
-“Can I solve the HVAC problem now without taking the entire cost at once?”
-I’d turn that into financing FAQs, same-day service posts, estimate follow-ups, objection responses and customer reactivation copy.
-Complete Same-Day Customer Growth Pack: $150 flat.
-Want two Therma Tech-specific samples first?</t>
-  </si>
-  <si>
-    <t>https://thermatechhvac.com/financing</t>
   </si>
   <si>
     <t>Script ID</t>
@@ -590,6 +599,9 @@
   </si>
   <si>
     <t>CostLess Heating &amp; Cooling</t>
+  </si>
+  <si>
+    <t>2026-09-06</t>
   </si>
   <si>
     <t>Los Gatos Roofing</t>
@@ -1339,19 +1351,19 @@
         <v>33</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N3" s="2" t="s">
         <v>27</v>
@@ -1365,10 +1377,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>17</v>
@@ -1377,26 +1389,28 @@
         <v>18</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H4" s="2"/>
+        <v>42</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="I4" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="N4" s="2" t="s">
         <v>27</v>
@@ -1410,38 +1424,40 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="H5" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>54</v>
+      </c>
       <c r="I5" s="2" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="N5" s="2" t="s">
         <v>27</v>
@@ -1455,38 +1471,38 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="N6" s="2" t="s">
         <v>27</v>
@@ -1500,38 +1516,38 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>67</v>
+        <v>17</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="N7" s="2" t="s">
         <v>27</v>
@@ -1545,40 +1561,38 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>80</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="H8" s="2"/>
       <c r="I8" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="N8" s="2" t="s">
         <v>27</v>
@@ -1592,38 +1606,38 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="N9" s="2" t="s">
         <v>27</v>
@@ -1637,10 +1651,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>17</v>
@@ -1649,26 +1663,26 @@
         <v>18</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="N10" s="2" t="s">
         <v>27</v>
@@ -1682,40 +1696,38 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>17</v>
+        <v>109</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>108</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="H11" s="2"/>
       <c r="I11" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N11" s="2" t="s">
         <v>27</v>
@@ -1760,142 +1772,142 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -1925,55 +1937,55 @@
   <sheetData>
     <row r="1" spans="1:17">
       <c r="A1" s="1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2" spans="1:17">
@@ -2043,18 +2055,18 @@
         <v>27</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:17">
       <c r="A4" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B4" s="2">
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -2078,18 +2090,18 @@
         <v>27</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B5" s="2">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -2113,18 +2125,18 @@
         <v>27</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" s="2" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B6" s="2">
         <v>5</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -2148,18 +2160,18 @@
         <v>27</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B7" s="2">
         <v>6</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
@@ -2183,18 +2195,18 @@
         <v>27</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B8" s="2">
         <v>7</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
@@ -2218,18 +2230,18 @@
         <v>27</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:17">
       <c r="A9" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B9" s="2">
         <v>8</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
@@ -2253,18 +2265,18 @@
         <v>27</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:17">
       <c r="A10" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B10" s="2">
         <v>9</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -2288,18 +2300,18 @@
         <v>27</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:17">
       <c r="A11" s="2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B11" s="2">
         <v>10</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -2323,7 +2335,7 @@
         <v>27</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -2371,30 +2383,30 @@
         <v>1</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="G1" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>170</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>28</v>
@@ -2408,13 +2420,13 @@
         <v>0</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>27</v>
+        <v>175</v>
       </c>
       <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="2" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>28</v>
@@ -2428,13 +2440,13 @@
         <v>0</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>27</v>
+        <v>175</v>
       </c>
       <c r="H3" s="2"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>28</v>
@@ -2448,13 +2460,13 @@
         <v>0</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>27</v>
+        <v>175</v>
       </c>
       <c r="H4" s="2"/>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>28</v>
@@ -2468,13 +2480,13 @@
         <v>0</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>27</v>
+        <v>175</v>
       </c>
       <c r="H5" s="2"/>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>28</v>
@@ -2488,13 +2500,13 @@
         <v>0</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>27</v>
+        <v>175</v>
       </c>
       <c r="H6" s="2"/>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>28</v>
@@ -2508,7 +2520,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>27</v>
+        <v>175</v>
       </c>
       <c r="H7" s="2"/>
     </row>
@@ -2540,10 +2552,10 @@
         <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -2560,7 +2572,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -2571,149 +2583,149 @@
         <v>31</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -2747,7 +2759,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="28" customHeight="1">
       <c r="A1" s="5" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -2756,17 +2768,17 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="1" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -2778,7 +2790,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="E4" s="3">
         <f>SUM(Pipeline!K:K)</f>
@@ -2787,14 +2799,14 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B5" s="2">
         <f>COUNTIF(Pipeline!J:J,"Contacted")</f>
         <v>0</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="E5" s="3">
         <f>SUM(Pipeline!L:L)</f>
@@ -2803,14 +2815,14 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B6" s="2">
         <f>COUNTIF(Pipeline!J:J,"Replied")</f>
         <v>0</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="E6" s="6">
         <f>IFERROR(COUNTIF(Pipeline!J:J,"Replied")/COUNTIF(Pipeline!D:D,"&lt;&gt;"),0)</f>
@@ -2819,14 +2831,14 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B7" s="2">
         <f>COUNTIF(Pipeline!J:J,"Negotiating")</f>
         <v>0</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="E7" s="6">
         <f>IFERROR(COUNTIF(Pipeline!J:J,"Won/Paid")/COUNTIF(Pipeline!D:D,"&lt;&gt;"),0)</f>
@@ -2835,7 +2847,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="B8" s="2">
         <f>COUNTIF(Pipeline!J:J,"Won/Paid")</f>
@@ -2844,7 +2856,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B9" s="2">
         <f>COUNTIF(Pipeline!J:J,"Fulfilled")</f>
@@ -2870,90 +2882,90 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -2972,19 +2984,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -3001,7 +3013,7 @@
         <v>6</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>